<commit_message>
changed mental for mental/cognitive + some cosmetic changes
</commit_message>
<xml_diff>
--- a/data/hypersomnolence_data_processed.xlsx
+++ b/data/hypersomnolence_data_processed.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vpmartin/Documents/VMBox/logi/content_analyses/hypersomnolence.content.analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097F81EA-6BDA-0D49-BC61-8B08914F8BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC498E90-FA33-2542-9DC3-C6EDE3779FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,13 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="96">
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Subcategory</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="97">
   <si>
     <t>Ab</t>
   </si>
@@ -308,6 +302,15 @@
   </si>
   <si>
     <t>Injury</t>
+  </si>
+  <si>
+    <t>Mental/cognitive symptoms</t>
+  </si>
+  <si>
+    <t>Dimension</t>
+  </si>
+  <si>
+    <t>Subdimension</t>
   </si>
 </sst>
 </file>
@@ -681,57 +684,57 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -763,16 +766,16 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -804,16 +807,16 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
         <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -845,16 +848,16 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
         <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" t="s">
-        <v>24</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -886,16 +889,16 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -927,16 +930,16 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -968,16 +971,16 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1009,16 +1012,16 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1050,16 +1053,16 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
         <v>35</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>37</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -1091,16 +1094,16 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -1132,16 +1135,16 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -1173,16 +1176,16 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1214,16 +1217,16 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -1255,16 +1258,16 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -1296,16 +1299,16 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -1337,16 +1340,16 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" t="s">
         <v>50</v>
-      </c>
-      <c r="C17" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" t="s">
-        <v>52</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -1378,16 +1381,16 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" t="s">
         <v>53</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>54</v>
-      </c>
-      <c r="C18" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" t="s">
-        <v>56</v>
       </c>
       <c r="E18">
         <v>2</v>
@@ -1419,16 +1422,16 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -1460,16 +1463,16 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" t="s">
         <v>59</v>
-      </c>
-      <c r="C20" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" t="s">
-        <v>61</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1501,16 +1504,16 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1542,16 +1545,16 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B22" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -1583,16 +1586,16 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" t="s">
         <v>66</v>
-      </c>
-      <c r="B23" t="s">
-        <v>66</v>
-      </c>
-      <c r="C23" t="s">
-        <v>67</v>
-      </c>
-      <c r="D23" t="s">
-        <v>68</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -1624,16 +1627,16 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -1665,16 +1668,16 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -1706,16 +1709,16 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B26" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C26" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -1747,16 +1750,16 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" t="s">
         <v>75</v>
-      </c>
-      <c r="C27" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" t="s">
-        <v>77</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -1788,16 +1791,16 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D28" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -1829,16 +1832,16 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D29" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1870,16 +1873,16 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -1911,16 +1914,16 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B31" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C31" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D31" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -1952,16 +1955,16 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C32" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D32" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -1993,16 +1996,16 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -2034,16 +2037,16 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" t="s">
         <v>90</v>
       </c>
-      <c r="B34" t="s">
+      <c r="D34" t="s">
         <v>91</v>
-      </c>
-      <c r="C34" t="s">
-        <v>92</v>
-      </c>
-      <c r="D34" t="s">
-        <v>93</v>
       </c>
       <c r="E34">
         <v>0</v>
@@ -2075,16 +2078,16 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B35" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C35" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D35" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E35">
         <v>0</v>
@@ -2116,5 +2119,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>